<commit_message>
Native-speaker confirmations for Noakhali, exact sentence matches from the research corpora with word-by-word boxes, Noakhali negative future rule
</commit_message>
<xml_diff>
--- a/database/reviewed/check_report.xlsx
+++ b/database/reviewed/check_report.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check report" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Check report'!$A$1:$H$248</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Check report'!$A$1:$H$255</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -31,7 +31,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +55,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="009BD8A8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
@@ -71,13 +76,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H248"/>
+  <dimension ref="A1:H255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4520,19 +4526,19 @@
           <t>আইঁ</t>
         </is>
       </c>
-      <c r="F100" s="3" t="inlineStr">
-        <is>
-          <t>Contradicted</t>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by native speaker</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>"আমি" in Noakhali data: 576x, as "আইঁ" 0x, most often "আই" (379x); "আইঁ" occurs 0x</t>
+          <t>"আমি" in Noakhali data: 576x, as "আইঁ" 0x, most often "আই" (379x); "আইঁ" occurs 0x; confirmed by Muskan (app owner)</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Dictionary only</t>
+          <t>Yes (native speaker)</t>
         </is>
       </c>
     </row>
@@ -4730,19 +4736,19 @@
           <t>হাল্লা</t>
         </is>
       </c>
-      <c r="F105" s="3" t="inlineStr">
-        <is>
-          <t>Contradicted</t>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by native speaker</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>"ভালো" in Noakhali data: 235x, as "হাল্লা" 0x, most often "ভালা" (144x); "হাল্লা" occurs 0x</t>
+          <t>"ভালো" in Noakhali data: 235x, as "হাল্লা" 0x, most often "ভালা" (144x); "হাল্লা" occurs 0x; confirmed by Muskan (app owner)</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Dictionary only</t>
+          <t>Dictionary (native speaker: real, but not the default)</t>
         </is>
       </c>
     </row>
@@ -4772,19 +4778,19 @@
           <t>ভালা</t>
         </is>
       </c>
-      <c r="F106" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by native speaker</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>"ভালো" in Noakhali data: 235x, as "ভালা" 144x, most often "ভালা" (144x); "ভালা" occurs 511x</t>
+          <t>"ভালো" in Noakhali data: 235x, as "ভালা" 144x, most often "ভালা" (144x); "ভালা" occurs 511x; confirmed by Muskan (app owner)</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes (native speaker)</t>
         </is>
       </c>
     </row>
@@ -4898,19 +4904,19 @@
           <t>হুত</t>
         </is>
       </c>
-      <c r="F109" s="3" t="inlineStr">
-        <is>
-          <t>Contradicted</t>
+      <c r="F109" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by native speaker</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>"ছেলে" in Noakhali data: 49x, as "হুত" 0x, most often "হোলা" (41x); "হুত" occurs 1x</t>
+          <t>"ছেলে" in Noakhali data: 49x, as "হুত" 0x, most often "হোলা" (41x); "হুত" occurs 1x; confirmed by Muskan (app owner)</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>Dictionary only</t>
+          <t>Yes (native speaker)</t>
         </is>
       </c>
     </row>
@@ -6576,7 +6582,7 @@
           <t>আমি</t>
         </is>
       </c>
-      <c r="F150" s="5" t="inlineStr">
+      <c r="F150" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -6614,7 +6620,7 @@
           <t>টাকা</t>
         </is>
       </c>
-      <c r="F151" s="5" t="inlineStr">
+      <c r="F151" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -6652,7 +6658,7 @@
           <t>টাহাঁ</t>
         </is>
       </c>
-      <c r="F152" s="5" t="inlineStr">
+      <c r="F152" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -6690,7 +6696,7 @@
           <t>আমি ভাত খামু।</t>
         </is>
       </c>
-      <c r="F153" s="5" t="inlineStr">
+      <c r="F153" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -6728,7 +6734,7 @@
           <t>আমি</t>
         </is>
       </c>
-      <c r="F154" s="5" t="inlineStr">
+      <c r="F154" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -6766,7 +6772,7 @@
           <t>আমী</t>
         </is>
       </c>
-      <c r="F155" s="5" t="inlineStr">
+      <c r="F155" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -6804,7 +6810,7 @@
           <t>ছেলে</t>
         </is>
       </c>
-      <c r="F156" s="5" t="inlineStr">
+      <c r="F156" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -6842,7 +6848,7 @@
           <t>ছাওয়াল</t>
         </is>
       </c>
-      <c r="F157" s="5" t="inlineStr">
+      <c r="F157" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -6880,7 +6886,7 @@
           <t>আমি ভাত খাবানে।</t>
         </is>
       </c>
-      <c r="F158" s="5" t="inlineStr">
+      <c r="F158" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -6918,7 +6924,7 @@
           <t>মুই</t>
         </is>
       </c>
-      <c r="F159" s="5" t="inlineStr">
+      <c r="F159" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -6956,7 +6962,7 @@
           <t>হামরা</t>
         </is>
       </c>
-      <c r="F160" s="5" t="inlineStr">
+      <c r="F160" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -6994,7 +7000,7 @@
           <t>ব্যাটা ছা</t>
         </is>
       </c>
-      <c r="F161" s="5" t="inlineStr">
+      <c r="F161" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -7032,7 +7038,7 @@
           <t>বেটি ছা</t>
         </is>
       </c>
-      <c r="F162" s="5" t="inlineStr">
+      <c r="F162" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -7070,7 +7076,7 @@
           <t>মুই ভাত খামো।</t>
         </is>
       </c>
-      <c r="F163" s="5" t="inlineStr">
+      <c r="F163" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -7108,7 +7114,7 @@
           <t>তুঁই কেমন আছেন?</t>
         </is>
       </c>
-      <c r="F164" s="5" t="inlineStr">
+      <c r="F164" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -7146,7 +7152,7 @@
           <t>বাহে কেমন আছেন?</t>
         </is>
       </c>
-      <c r="F165" s="5" t="inlineStr">
+      <c r="F165" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -7772,7 +7778,7 @@
           <t>ইঞ্জ</t>
         </is>
       </c>
-      <c r="F180" s="5" t="inlineStr">
+      <c r="F180" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -7810,7 +7816,7 @@
           <t>আম</t>
         </is>
       </c>
-      <c r="F181" s="5" t="inlineStr">
+      <c r="F181" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -7848,7 +7854,7 @@
           <t>দাকা</t>
         </is>
       </c>
-      <c r="F182" s="5" t="inlineStr">
+      <c r="F182" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -7886,7 +7892,7 @@
           <t>ইঞ্জ দাকাঞ্জ জমআ</t>
         </is>
       </c>
-      <c r="F183" s="5" t="inlineStr">
+      <c r="F183" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -7924,7 +7930,7 @@
           <t>চেলেকা মেনামা?</t>
         </is>
       </c>
-      <c r="F184" s="5" t="inlineStr">
+      <c r="F184" s="6" t="inlineStr">
         <is>
           <t>No data to check against</t>
         </is>
@@ -9412,19 +9418,19 @@
           <t>হুত</t>
         </is>
       </c>
-      <c r="F220" s="3" t="inlineStr">
-        <is>
-          <t>Contradicted</t>
+      <c r="F220" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by native speaker</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>"ছেলে" in Noakhali data: 49x, as "হুত" 0x, most often "হোলা" (41x); "হুত" occurs 1x</t>
+          <t>"ছেলে" in Noakhali data: 49x, as "হুত" 0x, most often "হোলা" (41x); "হুত" occurs 1x; confirmed by Muskan (app owner)</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>Dictionary only</t>
+          <t>Yes (native speaker)</t>
         </is>
       </c>
     </row>
@@ -9454,19 +9460,19 @@
           <t>ঝী</t>
         </is>
       </c>
-      <c r="F221" s="3" t="inlineStr">
-        <is>
-          <t>Contradicted</t>
+      <c r="F221" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by native speaker</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>"মেয়ে" in Noakhali data: 39x, as "ঝী" 0x, most often "মাইয়া" (30x); "ঝী" occurs 0x</t>
+          <t>"মেয়ে" in Noakhali data: 39x, as "ঝী" 0x, most often "মাইয়া" (30x); "ঝী" occurs 0x; confirmed by Muskan (app owner)</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>Dictionary only</t>
+          <t>Yes (native speaker)</t>
         </is>
       </c>
     </row>
@@ -10584,8 +10590,302 @@
         </is>
       </c>
     </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>native_confirmations.csv</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Noakhali</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>আমি</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>আইঁ</t>
+        </is>
+      </c>
+      <c r="F249" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by native speaker</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>"আমি" in Noakhali data: 576x, as "আইঁ" 0x, most often "আই" (379x); "আইঁ" occurs 0x; confirmed by Muskan (app owner)</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>Yes (native speaker)</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>native_confirmations.csv</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Noakhali</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>ছেলে</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>হুত</t>
+        </is>
+      </c>
+      <c r="F250" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by native speaker</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>"ছেলে" in Noakhali data: 49x, as "হুত" 0x, most often "হোলা" (41x); "হুত" occurs 1x; confirmed by Muskan (app owner)</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>Yes (native speaker)</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>native_confirmations.csv</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Noakhali</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>মেয়ে</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>ঝী</t>
+        </is>
+      </c>
+      <c r="F251" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by native speaker</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>"মেয়ে" in Noakhali data: 39x, as "ঝী" 0x, most often "মাইয়া" (30x); "ঝী" occurs 0x; confirmed by Muskan (app owner)</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>Yes (native speaker)</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>native_confirmations.csv</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Noakhali</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>ভালো</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>ভালা</t>
+        </is>
+      </c>
+      <c r="F252" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by native speaker</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>"ভালো" in Noakhali data: 235x, as "ভালা" 144x, most often "ভালা" (144x); "ভালা" occurs 511x; confirmed by Muskan (app owner)</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>Yes (native speaker)</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>native_confirmations.csv</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Noakhali</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>ভালো</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>হাল্লা</t>
+        </is>
+      </c>
+      <c r="F253" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by native speaker</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>"ভালো" in Noakhali data: 235x, as "হাল্লা" 0x, most often "ভালা" (144x); "হাল্লা" occurs 0x; confirmed by Muskan (app owner)</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>Dictionary (native speaker: real, but not the default)</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>native_confirmations.csv</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Noakhali</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>খাবো</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>খামু</t>
+        </is>
+      </c>
+      <c r="F254" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by native speaker</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>"খাবো" in Noakhali data: 9x, as "খামু" 0x, most often "খাইয়ুম" (7x); "খামু" occurs 4x; confirmed by Muskan (app owner)</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>Yes (native speaker)</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>native_confirmations.csv</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Noakhali</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Sentence</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>আমি ভাত খাবো না</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>আইঁ ভাত খাইতান ন</t>
+        </is>
+      </c>
+      <c r="F255" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by native speaker</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>confirmed by Muskan (app owner)</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>Yes (native speaker)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H248"/>
+  <autoFilter ref="A1:H255"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>